<commit_message>
Enhance chart and slide generation: - Added new fields to slide_info and build_slide functions for better data handling. - Improved chart data normalization and visibility checks in create_matplotlib_chart. - Updated JSON configurations for various charts to include new data points. - Refactored PDF and structure services for better data extraction and formatting. - Removed obsolete config files.
</commit_message>
<xml_diff>
--- a/data/config/common.xlsx
+++ b/data/config/common.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="83" documentId="11_33BF45607D3B04279C70531F978AA32C3F9FEA80" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A5ED1D8-A597-4437-B442-90D999C09DC0}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="11_33BF45607D3B04279C70531F978AA32C3F9FEA80" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{273C3E5A-55D0-4F20-8FD4-7CB474BA5070}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,7 +84,7 @@
     <t>rs</t>
   </si>
   <si>
-    <t>ps</t>
+    <t>pws</t>
   </si>
   <si>
     <t>guardia</t>
@@ -1140,7 +1140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1172,7 +1172,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1391,7 +1390,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AX1000"/>
+  <dimension ref="A1:AW1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.42578125" customWidth="1"/>
@@ -1419,7 +1418,7 @@
     <col min="30" max="42" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50">
+    <row r="1" spans="1:49">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1568,7 +1567,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:50" ht="409.6">
+    <row r="2" spans="1:49" ht="409.6">
       <c r="A2" s="3" t="s">
         <v>49</v>
       </c>
@@ -1716,9 +1715,8 @@
       <c r="AW2" t="s">
         <v>97</v>
       </c>
-      <c r="AX2" s="13"/>
-    </row>
-    <row r="3" spans="1:50">
+    </row>
+    <row r="3" spans="1:49">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1762,7 +1760,7 @@
       <c r="AO3" s="1"/>
       <c r="AP3" s="1"/>
     </row>
-    <row r="4" spans="1:50">
+    <row r="4" spans="1:49">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1806,7 +1804,7 @@
       <c r="AO4" s="1"/>
       <c r="AP4" s="1"/>
     </row>
-    <row r="5" spans="1:50">
+    <row r="5" spans="1:49">
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
@@ -1815,7 +1813,7 @@
       <c r="K5" s="5"/>
       <c r="AJ5" s="1"/>
     </row>
-    <row r="6" spans="1:50" ht="12.75">
+    <row r="6" spans="1:49" ht="12.75">
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
@@ -1823,7 +1821,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
     </row>
-    <row r="7" spans="1:50" ht="12.75">
+    <row r="7" spans="1:49" ht="12.75">
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
@@ -1831,7 +1829,7 @@
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
     </row>
-    <row r="8" spans="1:50" ht="12.75">
+    <row r="8" spans="1:49" ht="12.75">
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
@@ -1839,7 +1837,7 @@
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
     </row>
-    <row r="9" spans="1:50" ht="12.75">
+    <row r="9" spans="1:49" ht="12.75">
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
@@ -1847,7 +1845,7 @@
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
     </row>
-    <row r="10" spans="1:50" ht="12.75">
+    <row r="10" spans="1:49" ht="12.75">
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
@@ -1855,7 +1853,7 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
     </row>
-    <row r="11" spans="1:50" ht="12.75">
+    <row r="11" spans="1:49" ht="12.75">
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
@@ -1863,7 +1861,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
     </row>
-    <row r="12" spans="1:50" ht="12.75">
+    <row r="12" spans="1:49" ht="12.75">
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
@@ -1871,7 +1869,7 @@
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
     </row>
-    <row r="13" spans="1:50" ht="12.75">
+    <row r="13" spans="1:49" ht="12.75">
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
@@ -1879,7 +1877,7 @@
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
     </row>
-    <row r="14" spans="1:50" ht="12.75">
+    <row r="14" spans="1:49" ht="12.75">
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
@@ -1887,7 +1885,7 @@
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
     </row>
-    <row r="15" spans="1:50" ht="12.75">
+    <row r="15" spans="1:49" ht="12.75">
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
@@ -1895,7 +1893,7 @@
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
     </row>
-    <row r="16" spans="1:50" ht="12.75">
+    <row r="16" spans="1:49" ht="12.75">
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
@@ -9790,6 +9788,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1dac145f-12f1-46c0-a8b8-4af8e41b8063">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="00faf2f7-0679-4d56-a567-48d6a88ebe50" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101000848DB8A027FFA44ADDDDBDD228782A6" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="8d263d3cb1aa621d48e646d806cb1ef0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1dac145f-12f1-46c0-a8b8-4af8e41b8063" xmlns:ns3="00faf2f7-0679-4d56-a567-48d6a88ebe50" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="39e3593994817990d12a8ed679fcbd25" ns2:_="" ns3:_="">
     <xsd:import namespace="1dac145f-12f1-46c0-a8b8-4af8e41b8063"/>
@@ -9978,25 +9987,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1dac145f-12f1-46c0-a8b8-4af8e41b8063">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="00faf2f7-0679-4d56-a567-48d6a88ebe50" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56853F82-995A-4A3A-B277-F101D84DD634}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D04809AA-5BE2-4C64-8A16-01BE22A34EFF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4092DEF8-08CD-4356-8911-B29064BA7125}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4092DEF8-08CD-4356-8911-B29064BA7125}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D04809AA-5BE2-4C64-8A16-01BE22A34EFF}"/>
 </file>
</xml_diff>

<commit_message>
Agregar nuevas funcionalidades para convertir archivos XLSX a PDF y unir múltiples PDFs en un solo archivo
</commit_message>
<xml_diff>
--- a/data/config/common.xlsx
+++ b/data/config/common.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="99" documentId="11_33BF45607D3B04279C70531F978AA32C3F9FEA80" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C07ACCEE-E774-4C67-B3E8-80E581FE78A2}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="11_33BF45607D3B04279C70531F978AA32C3F9FEA80" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5CEC92B-8458-4213-9A36-7C11715CEE70}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -462,7 +462,7 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">AD Bridge:
@@ -471,7 +471,7 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t>Centraliza la autenticación y el inicio de sesión único (SSO) extendiendo Microsoft Active Directory a entornos Unix y Linux. Al unificar la gestión de identidades y políticas de grupo, elimina silos operativos y garantiza que las reglas de acceso y auditoría se apliquen de forma consistente en toda la infraestructura.</t>
@@ -482,7 +482,7 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">Endpoint Privilege Management (EPM-W):
@@ -491,7 +491,7 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t>Implementa el modelo de mínimo privilegio en Windows mediante la eliminación de administradores locales y la elevación dinámica de permisos solo para aplicaciones confiables. Mitiga riesgos de malware al controlar software no autorizado y ofrece trazabilidad total de actividades privilegiadas</t>
@@ -502,7 +502,7 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t>• Simulaciones (Simulations)</t>
@@ -510,7 +510,7 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t>: Motor de generación automática de campañas de phishing, smishing y robo de credenciales, diseñado para evaluar la vulnerabilidad real de los usuarios ante ataques de ingeniería social.</t>
@@ -799,7 +799,7 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">InvGate Service Desk:
@@ -808,7 +808,7 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">Permite una gobernanza total sobre las solicitudes mediante una configuración de permisos. Esto asegura que la información sensible, como los comentarios internos, solo sea visible para los perfiles técnicos adecuados, manteniendo la transparencia hacia el usuario final sin comprometer la privacidad operativa. Gracias a su motor de automatización y flujos de trabajo visuales, reducimos los tiempos de resolución y eliminamos los cuellos de botella.
@@ -820,19 +820,19 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>InvGate Asset Management:</t>
+      <t xml:space="preserve">InvGate Asset Management:
+</t>
     </r>
     <r>
       <rPr>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">
-Es el módulo de gestión de inventario y activos IT (hardware y software). Nos brinda visibilidad absoluta sobre la infraestructura, permitiendo un descubrimiento automático de activos y una gestión de inventarios en tiempo real.
+      <t xml:space="preserve">Es el módulo de gestión de inventario y activos IT (hardware y software). Nos brinda visibilidad absoluta sobre la infraestructura, permitiendo un descubrimiento automático de activos y una gestión de inventarios en tiempo real.
 </t>
     </r>
   </si>
@@ -1763,13 +1763,13 @@
       <c r="S2" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="T2" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="U2" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="V2" s="3" t="s">
+      <c r="V2" s="6" t="s">
         <v>75</v>
       </c>
       <c r="W2" s="3" t="s">
@@ -1814,10 +1814,10 @@
       <c r="AJ2" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="AK2" s="3" t="s">
+      <c r="AK2" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="AL2" s="3" t="s">
+      <c r="AL2" s="12" t="s">
         <v>91</v>
       </c>
       <c r="AM2" s="3" t="s">
@@ -9932,14 +9932,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1dac145f-12f1-46c0-a8b8-4af8e41b8063">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="00faf2f7-0679-4d56-a567-48d6a88ebe50" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10132,16 +10130,18 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1dac145f-12f1-46c0-a8b8-4af8e41b8063">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="00faf2f7-0679-4d56-a567-48d6a88ebe50" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4092DEF8-08CD-4356-8911-B29064BA7125}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56853F82-995A-4A3A-B277-F101D84DD634}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10149,5 +10149,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56853F82-995A-4A3A-B277-F101D84DD634}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4092DEF8-08CD-4356-8911-B29064BA7125}"/>
 </file>
</xml_diff>

<commit_message>
Add new PDF merging functionalities and update existing services
- Implemented endpoints for merging PDFs by order of payment and by specified names.
- Enhanced merge service to search and merge PDFs based on naming conventions.
- Updated PDF service to include new compatibility requirements.
</commit_message>
<xml_diff>
--- a/data/config/common.xlsx
+++ b/data/config/common.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="104" documentId="11_33BF45607D3B04279C70531F978AA32C3F9FEA80" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5CEC92B-8458-4213-9A36-7C11715CEE70}"/>
+  <xr:revisionPtr revIDLastSave="125" documentId="11_33BF45607D3B04279C70531F978AA32C3F9FEA80" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3907FCB-2D82-4AA3-9662-F115999BABCC}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="109">
   <si>
     <t>titulo</t>
   </si>
@@ -156,6 +156,9 @@
     <t>enc</t>
   </si>
   <si>
+    <t>fim</t>
+  </si>
+  <si>
     <t>iav</t>
   </si>
   <si>
@@ -175,9 +178,6 @@
   </si>
   <si>
     <t>tkd</t>
-  </si>
-  <si>
-    <t>fim</t>
   </si>
   <si>
     <t>sca</t>
@@ -841,7 +841,7 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t>• Detección de Vulnerabilidades:</t>
@@ -849,7 +849,7 @@
     <r>
       <rPr>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve"> Identifica de manera automática vulnerabilidades de software en los endpoints, cruzando el inventario de aplicaciones instaladas con bases de datos de CVE actualizadas.</t>
@@ -891,6 +891,25 @@
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve"> Módulo especializado en la generación de reportes y controles alineados con estándares internacionales como PCI DSS, GDPR, NIST 800-53 e HIPAA.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">• Monitoreo de Integridad de Archivos (FIM): </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Supervisa archivos y directorios críticos, detectando cambios no autorizados en atributos, contenidos o permisos para garantizar la trazabilidad de la información sensible.</t>
     </r>
   </si>
   <si>
@@ -1513,7 +1532,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.42578125" customWidth="1"/>
@@ -1538,10 +1557,12 @@
     <col min="26" max="26" width="24" customWidth="1"/>
     <col min="27" max="28" width="14.140625" customWidth="1"/>
     <col min="29" max="29" width="12.42578125" customWidth="1"/>
-    <col min="30" max="42" width="18.42578125" customWidth="1"/>
+    <col min="30" max="41" width="18.42578125" customWidth="1"/>
+    <col min="42" max="42" width="14.42578125" customWidth="1"/>
+    <col min="43" max="43" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54">
+    <row r="1" spans="1:55">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1668,7 +1689,7 @@
       <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
       <c r="AR1" t="s">
@@ -1690,22 +1711,25 @@
         <v>48</v>
       </c>
       <c r="AX1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AY1" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:54" ht="409.6">
+    <row r="2" spans="1:55" ht="409.6">
       <c r="A2" s="3" t="s">
         <v>54</v>
       </c>
@@ -1820,7 +1844,7 @@
       <c r="AL2" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="AM2" s="3" t="s">
+      <c r="AM2" s="6" t="s">
         <v>92</v>
       </c>
       <c r="AN2" s="3" t="s">
@@ -1829,25 +1853,25 @@
       <c r="AO2" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="AP2" s="6" t="s">
+      <c r="AP2" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="AQ2" s="9" t="s">
+      <c r="AQ2" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="AR2" s="10" t="s">
+      <c r="AR2" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="AS2" s="11" t="s">
+      <c r="AS2" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="AT2" s="8" t="s">
+      <c r="AT2" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="AU2" s="10" t="s">
+      <c r="AU2" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AV2" s="10" t="s">
         <v>101</v>
       </c>
       <c r="AW2" t="s">
@@ -1856,7 +1880,7 @@
       <c r="AX2" t="s">
         <v>103</v>
       </c>
-      <c r="AY2" s="13" t="s">
+      <c r="AY2" t="s">
         <v>104</v>
       </c>
       <c r="AZ2" s="13" t="s">
@@ -1868,8 +1892,11 @@
       <c r="BB2" s="13" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="3" spans="1:54">
+      <c r="BC2" s="13" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:55">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1912,8 +1939,9 @@
       <c r="AN3" s="1"/>
       <c r="AO3" s="1"/>
       <c r="AP3" s="1"/>
-    </row>
-    <row r="4" spans="1:54">
+      <c r="AQ3" s="1"/>
+    </row>
+    <row r="4" spans="1:55">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1956,8 +1984,9 @@
       <c r="AN4" s="1"/>
       <c r="AO4" s="1"/>
       <c r="AP4" s="1"/>
-    </row>
-    <row r="5" spans="1:54">
+      <c r="AQ4" s="1"/>
+    </row>
+    <row r="5" spans="1:55">
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
@@ -1966,7 +1995,7 @@
       <c r="K5" s="5"/>
       <c r="AJ5" s="1"/>
     </row>
-    <row r="6" spans="1:54" ht="12.75">
+    <row r="6" spans="1:55" ht="12.75">
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
@@ -1974,7 +2003,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
     </row>
-    <row r="7" spans="1:54" ht="12.75">
+    <row r="7" spans="1:55" ht="12.75">
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
@@ -1982,7 +2011,7 @@
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
     </row>
-    <row r="8" spans="1:54" ht="12.75">
+    <row r="8" spans="1:55" ht="12.75">
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
@@ -1990,7 +2019,7 @@
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
     </row>
-    <row r="9" spans="1:54" ht="12.75">
+    <row r="9" spans="1:55" ht="12.75">
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
@@ -1998,7 +2027,7 @@
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
     </row>
-    <row r="10" spans="1:54" ht="12.75">
+    <row r="10" spans="1:55" ht="12.75">
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
@@ -2006,7 +2035,7 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
     </row>
-    <row r="11" spans="1:54" ht="12.75">
+    <row r="11" spans="1:55" ht="12.75">
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
@@ -2014,7 +2043,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
     </row>
-    <row r="12" spans="1:54" ht="12.75">
+    <row r="12" spans="1:55" ht="12.75">
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
@@ -2022,7 +2051,7 @@
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
     </row>
-    <row r="13" spans="1:54" ht="12.75">
+    <row r="13" spans="1:55" ht="12.75">
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
@@ -2030,7 +2059,7 @@
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
     </row>
-    <row r="14" spans="1:54" ht="12.75">
+    <row r="14" spans="1:55" ht="12.75">
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
@@ -2038,7 +2067,7 @@
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
     </row>
-    <row r="15" spans="1:54" ht="12.75">
+    <row r="15" spans="1:55" ht="12.75">
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
@@ -2046,7 +2075,7 @@
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
     </row>
-    <row r="16" spans="1:54" ht="12.75">
+    <row r="16" spans="1:55" ht="12.75">
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
@@ -9932,12 +9961,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1dac145f-12f1-46c0-a8b8-4af8e41b8063">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="00faf2f7-0679-4d56-a567-48d6a88ebe50" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10130,18 +10161,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1dac145f-12f1-46c0-a8b8-4af8e41b8063">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="00faf2f7-0679-4d56-a567-48d6a88ebe50" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56853F82-995A-4A3A-B277-F101D84DD634}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4092DEF8-08CD-4356-8911-B29064BA7125}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10149,5 +10178,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4092DEF8-08CD-4356-8911-B29064BA7125}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56853F82-995A-4A3A-B277-F101D84DD634}"/>
 </file>
</xml_diff>